<commit_message>
Atualiza Gestão de Pendências · 2026-07-29T09:04:46.222-03:00
Responsável: Ana Paula da Mata Dias
</commit_message>
<xml_diff>
--- a/Base_Pendencias_FICO.xlsx
+++ b/Base_Pendencias_FICO.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\81063925\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://globalvale-my.sharepoint.com/personal/c0706142_vale_com/Documents/Arquivos de Chat do Microsoft Teams/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A6A02AB-2EB7-44B2-A1F8-27858C4205F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="97" documentId="13_ncr:1_{9A6A02AB-2EB7-44B2-A1F8-27858C4205F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9DDA87D0-3EF9-4733-9876-D3ED96BD8DFE}"/>
   <bookViews>
-    <workbookView xWindow="-75" yWindow="17880" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INSTRUCOES" sheetId="1" r:id="rId1"/>
@@ -20,8 +20,11 @@
     <sheet name="ALERTAS" sheetId="5" r:id="rId5"/>
     <sheet name="META" sheetId="6" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191028"/>
   <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -41,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="122">
   <si>
     <t>PAINEL DE PENDÊNCIAS FICO INFRA — BASE ÚNICA DE DADOS</t>
   </si>
@@ -148,6 +151,9 @@
     <t>Jul (4) + Ago (4) + Set (4) = 12 semanas</t>
   </si>
   <si>
+    <t>Mobilização crítica</t>
+  </si>
+  <si>
     <t>Marco final</t>
   </si>
   <si>
@@ -166,9 +172,6 @@
     <t>Jul (2) + Ago (4) + Set (4) = 10 semanas</t>
   </si>
   <si>
-    <t>Mobilização crítica</t>
-  </si>
-  <si>
     <t>Mobilização a partir de</t>
   </si>
   <si>
@@ -223,6 +226,9 @@
     <t>VALE</t>
   </si>
   <si>
+    <t>Em definição</t>
+  </si>
+  <si>
     <t>REPAROS</t>
   </si>
   <si>
@@ -253,57 +259,6 @@
     <t>SIM</t>
   </si>
   <si>
-    <t>65,5</t>
-  </si>
-  <si>
-    <t>13,1</t>
-  </si>
-  <si>
-    <t>32,8</t>
-  </si>
-  <si>
-    <t>6,6</t>
-  </si>
-  <si>
-    <t>21,8</t>
-  </si>
-  <si>
-    <t>4,4</t>
-  </si>
-  <si>
-    <t>16,4</t>
-  </si>
-  <si>
-    <t>3,3</t>
-  </si>
-  <si>
-    <t>2,6</t>
-  </si>
-  <si>
-    <t>41,7</t>
-  </si>
-  <si>
-    <t>8,3</t>
-  </si>
-  <si>
-    <t>20,8</t>
-  </si>
-  <si>
-    <t>4,2</t>
-  </si>
-  <si>
-    <t>13,9</t>
-  </si>
-  <si>
-    <t>2,8</t>
-  </si>
-  <si>
-    <t>10,4</t>
-  </si>
-  <si>
-    <t>2,1</t>
-  </si>
-  <si>
     <t>TITULO</t>
   </si>
   <si>
@@ -355,6 +310,15 @@
     <t>Divergência de baixas · VALE × EMPA</t>
   </si>
   <si>
+    <t xml:space="preserve">Controle VALE registra 99 baixadas. EMPA vai solicitar reinspeção de 140 pendências entre hoje e amanhã. </t>
+  </si>
+  <si>
+    <t>Gap crítico de mobilização — Pacote 01</t>
+  </si>
+  <si>
+    <t>EMPA com 12 colaboradores mobilizados frente aos 36 necessários (3 equipes × 12). Ritmo atual não zera as 749 pendências no prazo.</t>
+  </si>
+  <si>
     <t>Marcos contratuais · 15/10/2026</t>
   </si>
   <si>
@@ -427,6 +391,9 @@
     <t>DATA_REFERENCIA</t>
   </si>
   <si>
+    <t>07/07/2026</t>
+  </si>
+  <si>
     <t>CADENCIA</t>
   </si>
   <si>
@@ -436,28 +403,13 @@
     <t>PREMISSA</t>
   </si>
   <si>
+    <t>1 equipe com 12 colaboradores (1 encarregado + 4 oficiais + 8 serventes) executa em média 2 pendências/dia</t>
+  </si>
+  <si>
     <t>MARCO_FINAL</t>
   </si>
   <si>
     <t>15/10/2026 — Hidro e TAC 05 (Pacote 01)</t>
-  </si>
-  <si>
-    <t>Em definição</t>
-  </si>
-  <si>
-    <t>Gap crítico de mobilização — Pacote 01</t>
-  </si>
-  <si>
-    <t>EMPA com 12 colaboradores mobilizados frente aos 36 necessários (3 equipes × 12). Ritmo atual não zera as 749 pendências no prazo.</t>
-  </si>
-  <si>
-    <t>1 equipe com 12 colaboradores (1 encarregado + 4 oficiais + 8 serventes) executa em média 2 pendências/dia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Controle VALE registra 99 baixadas. EMPA vai solicitar reinspeção de 140 pendências entre hoje e amanhã. </t>
-  </si>
-  <si>
-    <t>07/07/2026</t>
   </si>
 </sst>
 </file>
@@ -605,7 +557,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -646,6 +598,15 @@
     </xf>
     <xf numFmtId="14" fontId="6" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -730,6 +691,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -912,95 +877,95 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:B20"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
     <col min="2" max="2" width="115" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:2" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:2" ht="20" x14ac:dyDescent="0.4">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B3" s="2"/>
     </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B5" s="2"/>
     </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B6" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B7" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B8" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B9" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B10" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B11" s="2"/>
     </row>
-    <row r="12" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B12" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B13" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B14" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B15" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B16" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B17" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B18" s="2"/>
     </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B19" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B20" s="2" t="s">
         <v>14</v>
       </c>
@@ -1014,26 +979,27 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:P4"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="2" width="11" customWidth="1"/>
-    <col min="3" max="3" width="20" customWidth="1"/>
-    <col min="4" max="4" width="34" customWidth="1"/>
-    <col min="5" max="5" width="13" customWidth="1"/>
-    <col min="6" max="6" width="9" customWidth="1"/>
-    <col min="7" max="7" width="10" customWidth="1"/>
-    <col min="8" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="9" customWidth="1"/>
-    <col min="11" max="11" width="17" customWidth="1"/>
-    <col min="12" max="12" width="7" customWidth="1"/>
-    <col min="13" max="13" width="13" customWidth="1"/>
-    <col min="14" max="14" width="20" customWidth="1"/>
-    <col min="15" max="15" width="14" customWidth="1"/>
-    <col min="16" max="16" width="55" customWidth="1"/>
+    <col min="1" max="1" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.08984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.36328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.08984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.7265625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.1796875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="19.1796875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.6328125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="44.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" ht="27" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>15</v>
       </c>
@@ -1083,7 +1049,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" ht="25" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
         <v>31</v>
       </c>
@@ -1117,7 +1083,7 @@
         <v>67</v>
       </c>
       <c r="K2" s="7" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="L2" s="8">
         <v>15</v>
@@ -1126,25 +1092,25 @@
         <v>0</v>
       </c>
       <c r="N2" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="O2" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="P2" s="7"/>
     </row>
-    <row r="3" spans="1:16" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" ht="25" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E3" s="8">
         <v>1</v>
@@ -1166,7 +1132,7 @@
         <v>50</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="L3" s="8">
         <v>20</v>
@@ -1184,7 +1150,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" ht="25" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
         <v>45</v>
       </c>
@@ -1242,18 +1208,18 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9" customWidth="1"/>
-    <col min="2" max="2" width="11" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="11" customWidth="1"/>
-    <col min="7" max="7" width="42" customWidth="1"/>
+    <col min="1" max="1" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.6328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.6328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="30.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>15</v>
       </c>
@@ -1276,7 +1242,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
         <v>31</v>
       </c>
@@ -1287,18 +1253,18 @@
         <v>56</v>
       </c>
       <c r="D2" s="6">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E2" s="8">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F2" s="10">
         <f t="shared" ref="F2:F11" si="0">D2-E2</f>
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="G2" s="7"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
         <v>31</v>
       </c>
@@ -1309,20 +1275,20 @@
         <v>57</v>
       </c>
       <c r="D3" s="6">
-        <v>80</v>
+        <v>111</v>
       </c>
       <c r="E3" s="8">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F3" s="10">
         <f t="shared" si="0"/>
-        <v>77</v>
+        <v>103</v>
       </c>
       <c r="G3" s="7" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
         <v>31</v>
       </c>
@@ -1333,20 +1299,20 @@
         <v>59</v>
       </c>
       <c r="D4" s="6">
-        <v>78</v>
+        <v>97</v>
       </c>
       <c r="E4" s="8">
         <v>0</v>
       </c>
       <c r="F4" s="10">
         <f t="shared" si="0"/>
-        <v>78</v>
+        <v>97</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
         <v>31</v>
       </c>
@@ -1354,37 +1320,35 @@
         <v>32</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D5" s="6">
-        <f>848-78-84-80</f>
-        <v>606</v>
+        <v>83</v>
       </c>
       <c r="E5" s="8">
-        <f>99-29-3</f>
-        <v>67</v>
+        <v>26</v>
       </c>
       <c r="F5" s="10">
         <f t="shared" si="0"/>
-        <v>539</v>
+        <v>57</v>
       </c>
       <c r="G5" s="7"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C6" s="7" t="s">
         <v>56</v>
       </c>
       <c r="D6" s="6">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="E6" s="8">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="F6" s="10">
         <f t="shared" si="0"/>
@@ -1392,21 +1356,21 @@
       </c>
       <c r="G6" s="7"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C7" s="7" t="s">
         <v>57</v>
       </c>
       <c r="D7" s="6">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E7" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7" s="10">
         <f t="shared" si="0"/>
@@ -1414,100 +1378,96 @@
       </c>
       <c r="G7" s="7"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D8" s="6">
-        <f>727-53-40</f>
-        <v>634</v>
+        <v>114</v>
       </c>
       <c r="E8" s="8">
-        <f>50-25-1</f>
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="F8" s="10">
         <f t="shared" si="0"/>
-        <v>610</v>
+        <v>95</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="D9" s="6">
-        <v>37</v>
+      <c r="D9" s="17">
+        <v>33</v>
       </c>
       <c r="E9" s="8">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F9" s="10">
         <f t="shared" si="0"/>
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G9" s="7"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A10" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="D10" s="6">
-        <v>72</v>
+      <c r="D10" s="17">
+        <v>50</v>
       </c>
       <c r="E10" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F10" s="10">
         <f t="shared" si="0"/>
-        <v>71</v>
+        <v>48</v>
       </c>
       <c r="G10" s="7"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="C11" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="D11" s="6">
-        <f>595-37-72</f>
-        <v>486</v>
+      <c r="C11" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="D11" s="17">
+        <v>45</v>
       </c>
       <c r="E11" s="8">
-        <f>56-3-1</f>
-        <v>52</v>
+        <v>12</v>
       </c>
       <c r="F11" s="10">
         <f t="shared" si="0"/>
-        <v>434</v>
+        <v>33</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -1518,79 +1478,79 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:H13"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9" customWidth="1"/>
-    <col min="2" max="2" width="11" customWidth="1"/>
-    <col min="3" max="3" width="13" customWidth="1"/>
-    <col min="4" max="4" width="11" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="9" customWidth="1"/>
-    <col min="7" max="7" width="12" customWidth="1"/>
-    <col min="8" max="8" width="32" customWidth="1"/>
+    <col min="1" max="1" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.08984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>15</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>23</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
         <v>31</v>
       </c>
       <c r="B2" s="10">
         <v>1</v>
       </c>
-      <c r="C2" s="6">
-        <v>39.799999999999997</v>
-      </c>
-      <c r="D2" s="6">
-        <v>8</v>
+      <c r="C2" s="19">
+        <v>6.5555555555555554</v>
+      </c>
+      <c r="D2" s="19">
+        <v>1.3111111111111111</v>
       </c>
       <c r="E2" s="6">
         <v>12</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G2" s="6"/>
       <c r="H2" s="7"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
         <v>31</v>
       </c>
       <c r="B3" s="10">
         <v>2</v>
       </c>
-      <c r="C3" s="6">
-        <v>19.899999999999999</v>
-      </c>
-      <c r="D3" s="6">
-        <v>4</v>
+      <c r="C3" s="19">
+        <v>11.444444444444445</v>
+      </c>
+      <c r="D3" s="19">
+        <v>2.2888888888888888</v>
       </c>
       <c r="E3" s="6">
         <v>24</v>
@@ -1599,40 +1559,40 @@
       <c r="G3" s="6"/>
       <c r="H3" s="7"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
         <v>31</v>
       </c>
       <c r="B4" s="10">
         <v>3</v>
       </c>
-      <c r="C4" s="6">
-        <v>13.3</v>
-      </c>
-      <c r="D4" s="6">
-        <v>2.7</v>
+      <c r="C4" s="19">
+        <v>10.777777777777779</v>
+      </c>
+      <c r="D4" s="19">
+        <v>2.1555555555555559</v>
       </c>
       <c r="E4" s="6">
         <v>36</v>
       </c>
       <c r="F4" s="6"/>
       <c r="G4" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H4" s="7"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="B5" s="10">
         <v>1</v>
       </c>
-      <c r="C5" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>71</v>
+      <c r="C5" s="19">
+        <v>6.333333333333333</v>
+      </c>
+      <c r="D5" s="19">
+        <v>1.2666666666666666</v>
       </c>
       <c r="E5" s="6">
         <v>12</v>
@@ -1641,18 +1601,18 @@
       <c r="G5" s="6"/>
       <c r="H5" s="7"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B6" s="10">
         <v>2</v>
       </c>
-      <c r="C6" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>73</v>
+      <c r="C6" s="19">
+        <v>3.1111111111111112</v>
+      </c>
+      <c r="D6" s="19">
+        <v>0.62222222222222223</v>
       </c>
       <c r="E6" s="6">
         <v>24</v>
@@ -1661,40 +1621,40 @@
       <c r="G6" s="6"/>
       <c r="H6" s="7"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B7" s="10">
         <v>3</v>
       </c>
-      <c r="C7" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>75</v>
+      <c r="C7" s="19">
+        <v>4.333333333333333</v>
+      </c>
+      <c r="D7" s="19">
+        <v>0.86666666666666659</v>
       </c>
       <c r="E7" s="6">
         <v>36</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G7" s="6"/>
       <c r="H7" s="7"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B8" s="10">
         <v>4</v>
       </c>
-      <c r="C8" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>77</v>
+      <c r="C8" s="19">
+        <v>10.555555555555555</v>
+      </c>
+      <c r="D8" s="19">
+        <v>2.1111111111111112</v>
       </c>
       <c r="E8" s="6">
         <v>48</v>
@@ -1703,40 +1663,40 @@
       <c r="G8" s="6"/>
       <c r="H8" s="7"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B9" s="10">
         <v>5</v>
       </c>
-      <c r="C9" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>78</v>
+      <c r="C9" s="19">
+        <v>3.6666666666666665</v>
+      </c>
+      <c r="D9" s="19">
+        <v>0.73333333333333328</v>
       </c>
       <c r="E9" s="6">
         <v>60</v>
       </c>
       <c r="F9" s="6"/>
       <c r="G9" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H9" s="7"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="6" t="s">
         <v>45</v>
       </c>
       <c r="B10" s="10">
         <v>1</v>
       </c>
-      <c r="C10" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>80</v>
+      <c r="C10" s="19">
+        <v>5.333333333333333</v>
+      </c>
+      <c r="D10" s="19">
+        <v>1.0666666666666667</v>
       </c>
       <c r="E10" s="6">
         <v>12</v>
@@ -1745,18 +1705,18 @@
       <c r="G10" s="6"/>
       <c r="H10" s="7"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
         <v>45</v>
       </c>
       <c r="B11" s="10">
         <v>2</v>
       </c>
-      <c r="C11" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>82</v>
+      <c r="C11" s="19">
+        <v>3.6666666666666665</v>
+      </c>
+      <c r="D11" s="19">
+        <v>0.73333333333333328</v>
       </c>
       <c r="E11" s="6">
         <v>24</v>
@@ -1764,50 +1724,6 @@
       <c r="F11" s="6"/>
       <c r="G11" s="6"/>
       <c r="H11" s="7"/>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="B12" s="10">
-        <v>3</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="E12" s="6">
-        <v>36</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="G12" s="6"/>
-      <c r="H12" s="7"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="B13" s="10">
-        <v>4</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="E13" s="6">
-        <v>48</v>
-      </c>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="H13" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1818,15 +1734,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9" customWidth="1"/>
-    <col min="2" max="2" width="11" customWidth="1"/>
-    <col min="3" max="3" width="42" customWidth="1"/>
-    <col min="4" max="4" width="85" customWidth="1"/>
+    <col min="1" max="1" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="84.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>15</v>
       </c>
@@ -1834,234 +1750,234 @@
         <v>51</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>87</v>
+        <v>71</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="25" x14ac:dyDescent="0.35">
       <c r="A2" s="10" t="s">
-        <v>89</v>
+        <v>73</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>90</v>
+        <v>74</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>91</v>
+        <v>75</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="25" x14ac:dyDescent="0.35">
       <c r="A3" s="10" t="s">
-        <v>89</v>
+        <v>73</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="25" x14ac:dyDescent="0.35">
       <c r="A4" s="10" t="s">
-        <v>89</v>
+        <v>73</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="25" x14ac:dyDescent="0.35">
       <c r="A5" s="10" t="s">
-        <v>89</v>
+        <v>73</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="25" x14ac:dyDescent="0.35">
       <c r="A6" s="10" t="s">
         <v>31</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="25" x14ac:dyDescent="0.35">
       <c r="A7" s="10" t="s">
         <v>31</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="25" x14ac:dyDescent="0.35">
       <c r="A8" s="10" t="s">
         <v>31</v>
       </c>
       <c r="B8" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="D8" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="C8" s="12" t="s">
-        <v>134</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="10" t="s">
         <v>31</v>
       </c>
       <c r="B9" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="25" x14ac:dyDescent="0.35">
+      <c r="A10" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="25" x14ac:dyDescent="0.35">
+      <c r="A11" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="D11" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="C9" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="B10" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="C10" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A11" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="B11" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="C11" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:4" ht="25" x14ac:dyDescent="0.35">
       <c r="A12" s="10" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>110</v>
+        <v>97</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="10" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>90</v>
+        <v>74</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="25" x14ac:dyDescent="0.35">
       <c r="A14" s="10" t="s">
         <v>45</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>114</v>
+        <v>101</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="10" t="s">
         <v>45</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>116</v>
+        <v>103</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="10" t="s">
         <v>45</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>90</v>
+        <v>74</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>118</v>
+        <v>105</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="25" x14ac:dyDescent="0.35">
       <c r="A17" s="10" t="s">
         <v>45</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>120</v>
+        <v>107</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -2073,66 +1989,66 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
-        <v>122</v>
+        <v>109</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="15" t="s">
-        <v>87</v>
+        <v>71</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="15" t="s">
-        <v>125</v>
+        <v>112</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" s="15" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="15" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="25" x14ac:dyDescent="0.35">
       <c r="A6" s="15" t="s">
-        <v>130</v>
+        <v>118</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" s="15" t="s">
-        <v>131</v>
+        <v>120</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>132</v>
+        <v>121</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza Gestão de Pendências · 2026-08-04T07:57:12.260-03:00
Responsável: Ana Paula da Mata Dias
</commit_message>
<xml_diff>
--- a/Base_Pendencias_FICO.xlsx
+++ b/Base_Pendencias_FICO.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://globalvale-my.sharepoint.com/personal/c0706142_vale_com/Documents/Arquivos de Chat do Microsoft Teams/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://globalvale.sharepoint.com/sites/PlanejamentoFICO/Shared Documents/General/04. Rotinas de desempenho FICO/06_Central de Acesso - Atualização/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="97" documentId="13_ncr:1_{9A6A02AB-2EB7-44B2-A1F8-27858C4205F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9DDA87D0-3EF9-4733-9876-D3ED96BD8DFE}"/>
+  <xr:revisionPtr revIDLastSave="119" documentId="13_ncr:1_{9A6A02AB-2EB7-44B2-A1F8-27858C4205F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E4681AB2-670D-4289-A271-DBFDD627E6B6}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INSTRUCOES" sheetId="1" r:id="rId1"/>
@@ -429,67 +429,67 @@
       <sz val="16"/>
       <color rgb="FF142A4C"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF333333"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF142A4C"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFF89B32"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="7">
@@ -557,7 +557,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -597,12 +597,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="6" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -691,10 +685,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -877,95 +867,95 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:B20"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
     <col min="2" max="2" width="115" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:2" ht="20" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:2" ht="21" x14ac:dyDescent="0.4">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B3" s="2"/>
     </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B5" s="2"/>
     </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B6" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B7" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B8" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B9" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B10" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B11" s="2"/>
     </row>
-    <row r="12" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B12" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B13" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B14" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B15" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B16" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B17" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B18" s="2"/>
     </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B19" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B20" s="2" t="s">
         <v>14</v>
       </c>
@@ -979,27 +969,27 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:P4"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.6328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.08984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.08984375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.36328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.44140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.08984375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.36328125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.7265625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="5.1796875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="17.453125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="19.1796875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.6328125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="44.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="19.109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="44.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="27" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>15</v>
       </c>
@@ -1049,7 +1039,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="25" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
         <v>31</v>
       </c>
@@ -1099,7 +1089,7 @@
       </c>
       <c r="P2" s="7"/>
     </row>
-    <row r="3" spans="1:16" ht="25" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>38</v>
       </c>
@@ -1150,7 +1140,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="25" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
         <v>45</v>
       </c>
@@ -1208,18 +1198,18 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.6328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.6328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="30.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="32.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>15</v>
       </c>
@@ -1242,7 +1232,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
         <v>31</v>
       </c>
@@ -1256,15 +1246,15 @@
         <v>86</v>
       </c>
       <c r="E2" s="8">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="F2" s="10">
         <f t="shared" ref="F2:F11" si="0">D2-E2</f>
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="G2" s="7"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>31</v>
       </c>
@@ -1278,17 +1268,17 @@
         <v>111</v>
       </c>
       <c r="E3" s="8">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F3" s="10">
         <f t="shared" si="0"/>
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="G3" s="7" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
         <v>31</v>
       </c>
@@ -1299,20 +1289,20 @@
         <v>59</v>
       </c>
       <c r="D4" s="6">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="E4" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4" s="10">
         <f t="shared" si="0"/>
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="G4" s="7" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
         <v>31</v>
       </c>
@@ -1326,15 +1316,15 @@
         <v>83</v>
       </c>
       <c r="E5" s="8">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="F5" s="10">
         <f t="shared" si="0"/>
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="G5" s="7"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
         <v>38</v>
       </c>
@@ -1356,7 +1346,7 @@
       </c>
       <c r="G6" s="7"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>38</v>
       </c>
@@ -1370,15 +1360,15 @@
         <v>39</v>
       </c>
       <c r="E7" s="8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F7" s="10">
         <f t="shared" si="0"/>
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="G7" s="7"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>38</v>
       </c>
@@ -1392,49 +1382,49 @@
         <v>114</v>
       </c>
       <c r="E8" s="8">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="F8" s="10">
         <f t="shared" si="0"/>
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="G8" s="7" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A9" s="17" t="s">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="D9" s="17">
+      <c r="D9" s="6">
         <v>33</v>
       </c>
       <c r="E9" s="8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F9" s="10">
         <f t="shared" si="0"/>
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="G9" s="7"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A10" s="17" t="s">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="C10" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="D10" s="17">
+      <c r="D10" s="6">
         <v>50</v>
       </c>
       <c r="E10" s="8">
@@ -1446,25 +1436,25 @@
       </c>
       <c r="G10" s="7"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A11" s="17" t="s">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="C11" s="18" t="s">
+      <c r="C11" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="D11" s="17">
+      <c r="D11" s="6">
         <v>45</v>
       </c>
       <c r="E11" s="8">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F11" s="10">
         <f t="shared" si="0"/>
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G11" s="7" t="s">
         <v>63</v>
@@ -1479,19 +1469,19 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.08984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.08984375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>15</v>
       </c>
@@ -1517,18 +1507,18 @@
         <v>69</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
         <v>31</v>
       </c>
       <c r="B2" s="10">
         <v>1</v>
       </c>
-      <c r="C2" s="19">
-        <v>6.5555555555555554</v>
-      </c>
-      <c r="D2" s="19">
-        <v>1.3111111111111111</v>
+      <c r="C2" s="17">
+        <v>5.375</v>
+      </c>
+      <c r="D2" s="17">
+        <v>1.075</v>
       </c>
       <c r="E2" s="6">
         <v>12</v>
@@ -1539,18 +1529,18 @@
       <c r="G2" s="6"/>
       <c r="H2" s="7"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>31</v>
       </c>
       <c r="B3" s="10">
         <v>2</v>
       </c>
-      <c r="C3" s="19">
-        <v>11.444444444444445</v>
-      </c>
-      <c r="D3" s="19">
-        <v>2.2888888888888888</v>
+      <c r="C3" s="17">
+        <v>12.625</v>
+      </c>
+      <c r="D3" s="17">
+        <v>2.5249999999999999</v>
       </c>
       <c r="E3" s="6">
         <v>24</v>
@@ -1559,18 +1549,18 @@
       <c r="G3" s="6"/>
       <c r="H3" s="7"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
         <v>31</v>
       </c>
       <c r="B4" s="10">
         <v>3</v>
       </c>
-      <c r="C4" s="19">
-        <v>10.777777777777779</v>
-      </c>
-      <c r="D4" s="19">
-        <v>2.1555555555555559</v>
+      <c r="C4" s="17">
+        <v>12.5</v>
+      </c>
+      <c r="D4" s="17">
+        <v>2.5</v>
       </c>
       <c r="E4" s="6">
         <v>36</v>
@@ -1581,18 +1571,18 @@
       </c>
       <c r="H4" s="7"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
         <v>31</v>
       </c>
       <c r="B5" s="10">
         <v>1</v>
       </c>
-      <c r="C5" s="19">
-        <v>6.333333333333333</v>
-      </c>
-      <c r="D5" s="19">
-        <v>1.2666666666666666</v>
+      <c r="C5" s="17">
+        <v>6</v>
+      </c>
+      <c r="D5" s="17">
+        <v>1.2</v>
       </c>
       <c r="E5" s="6">
         <v>12</v>
@@ -1601,18 +1591,18 @@
       <c r="G5" s="6"/>
       <c r="H5" s="7"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
         <v>38</v>
       </c>
       <c r="B6" s="10">
         <v>2</v>
       </c>
-      <c r="C6" s="19">
-        <v>3.1111111111111112</v>
-      </c>
-      <c r="D6" s="19">
-        <v>0.62222222222222223</v>
+      <c r="C6" s="17">
+        <v>3.5</v>
+      </c>
+      <c r="D6" s="17">
+        <v>0.7</v>
       </c>
       <c r="E6" s="6">
         <v>24</v>
@@ -1621,18 +1611,18 @@
       <c r="G6" s="6"/>
       <c r="H6" s="7"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>38</v>
       </c>
       <c r="B7" s="10">
         <v>3</v>
       </c>
-      <c r="C7" s="19">
-        <v>4.333333333333333</v>
-      </c>
-      <c r="D7" s="19">
-        <v>0.86666666666666659</v>
+      <c r="C7" s="17">
+        <v>4.625</v>
+      </c>
+      <c r="D7" s="17">
+        <v>0.92500000000000004</v>
       </c>
       <c r="E7" s="6">
         <v>36</v>
@@ -1643,18 +1633,18 @@
       <c r="G7" s="6"/>
       <c r="H7" s="7"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>38</v>
       </c>
       <c r="B8" s="10">
         <v>4</v>
       </c>
-      <c r="C8" s="19">
-        <v>10.555555555555555</v>
-      </c>
-      <c r="D8" s="19">
-        <v>2.1111111111111112</v>
+      <c r="C8" s="17">
+        <v>11.375</v>
+      </c>
+      <c r="D8" s="17">
+        <v>2.2749999999999999</v>
       </c>
       <c r="E8" s="6">
         <v>48</v>
@@ -1663,18 +1653,18 @@
       <c r="G8" s="6"/>
       <c r="H8" s="7"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
         <v>45</v>
       </c>
       <c r="B9" s="10">
         <v>5</v>
       </c>
-      <c r="C9" s="19">
-        <v>3.6666666666666665</v>
-      </c>
-      <c r="D9" s="19">
-        <v>0.73333333333333328</v>
+      <c r="C9" s="17">
+        <v>3.875</v>
+      </c>
+      <c r="D9" s="17">
+        <v>0.77500000000000002</v>
       </c>
       <c r="E9" s="6">
         <v>60</v>
@@ -1685,18 +1675,18 @@
       </c>
       <c r="H9" s="7"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
         <v>45</v>
       </c>
       <c r="B10" s="10">
         <v>1</v>
       </c>
-      <c r="C10" s="19">
-        <v>5.333333333333333</v>
-      </c>
-      <c r="D10" s="19">
-        <v>1.0666666666666667</v>
+      <c r="C10" s="17">
+        <v>6</v>
+      </c>
+      <c r="D10" s="17">
+        <v>1.2</v>
       </c>
       <c r="E10" s="6">
         <v>12</v>
@@ -1705,18 +1695,18 @@
       <c r="G10" s="6"/>
       <c r="H10" s="7"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
         <v>45</v>
       </c>
       <c r="B11" s="10">
         <v>2</v>
       </c>
-      <c r="C11" s="19">
-        <v>3.6666666666666665</v>
-      </c>
-      <c r="D11" s="19">
-        <v>0.73333333333333328</v>
+      <c r="C11" s="17">
+        <v>4</v>
+      </c>
+      <c r="D11" s="17">
+        <v>0.8</v>
       </c>
       <c r="E11" s="6">
         <v>24</v>
@@ -1734,15 +1724,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="38.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="84.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="84.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>15</v>
       </c>
@@ -1756,7 +1746,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="25" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
         <v>73</v>
       </c>
@@ -1770,7 +1760,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="25" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
         <v>73</v>
       </c>
@@ -1784,7 +1774,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="25" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
         <v>73</v>
       </c>
@@ -1798,7 +1788,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="25" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
         <v>73</v>
       </c>
@@ -1812,7 +1802,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="25" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
         <v>31</v>
       </c>
@@ -1826,7 +1816,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="25" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="s">
         <v>31</v>
       </c>
@@ -1840,7 +1830,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="25" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A8" s="10" t="s">
         <v>31</v>
       </c>
@@ -1854,7 +1844,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="10" t="s">
         <v>31</v>
       </c>
@@ -1868,7 +1858,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="25" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A10" s="10" t="s">
         <v>38</v>
       </c>
@@ -1882,7 +1872,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="25" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
         <v>38</v>
       </c>
@@ -1896,7 +1886,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="25" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A12" s="10" t="s">
         <v>38</v>
       </c>
@@ -1910,7 +1900,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A13" s="10" t="s">
         <v>38</v>
       </c>
@@ -1924,7 +1914,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="25" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A14" s="10" t="s">
         <v>45</v>
       </c>
@@ -1938,7 +1928,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A15" s="10" t="s">
         <v>45</v>
       </c>
@@ -1952,7 +1942,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A16" s="10" t="s">
         <v>45</v>
       </c>
@@ -1966,7 +1956,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="25" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A17" s="10" t="s">
         <v>45</v>
       </c>
@@ -1989,13 +1979,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>109</v>
       </c>
@@ -2003,7 +1993,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="15" t="s">
         <v>71</v>
       </c>
@@ -2011,7 +2001,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="15" t="s">
         <v>112</v>
       </c>
@@ -2019,7 +2009,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="15" t="s">
         <v>114</v>
       </c>
@@ -2027,7 +2017,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="15" t="s">
         <v>116</v>
       </c>
@@ -2035,7 +2025,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="25" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A6" s="15" t="s">
         <v>118</v>
       </c>
@@ -2043,7 +2033,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="15" t="s">
         <v>120</v>
       </c>
@@ -2055,6 +2045,339 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100401A7D55F60B18408D7825C28E029F51" ma:contentTypeVersion="19" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="26245b19684232a249215bac47317027">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="b633a64c-250e-4f9b-b03e-91a68bc51404" xmlns:ns3="442af37a-3796-4d85-82a9-7fed4a3d9bab" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0b8051d1477f5ab751da8276506a6b46" ns1:_="" ns2:_="" ns3:_="">
+    <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
+    <xsd:import namespace="b633a64c-250e-4f9b-b03e-91a68bc51404"/>
+    <xsd:import namespace="442af37a-3796-4d85-82a9-7fed4a3d9bab"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns1:_ip_UnifiedCompliancePolicyProperties" minOccurs="0"/>
+                <xsd:element ref="ns1:_ip_UnifiedCompliancePolicyUIAction" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns2:_Flow_SignoffStatus" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="http://schemas.microsoft.com/sharepoint/v3" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="_ip_UnifiedCompliancePolicyProperties" ma:index="18" nillable="true" ma:displayName="Propriedades da Política de Conformidade Unificada" ma:hidden="true" ma:internalName="_ip_UnifiedCompliancePolicyProperties">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="_ip_UnifiedCompliancePolicyUIAction" ma:index="19" nillable="true" ma:displayName="Ação de Interface do Usuário da Política de Conformidade Unificada" ma:hidden="true" ma:internalName="_ip_UnifiedCompliancePolicyUIAction">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b633a64c-250e-4f9b-b03e-91a68bc51404" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="11" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Marcações de imagem" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="7bfb4e49-6f5d-460f-8245-f0e15177ea6b" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="13" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="14" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="15" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="20" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="21" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="22" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="_Flow_SignoffStatus" ma:index="23" nillable="true" ma:displayName="Sign-off status" ma:internalName="Sign_x002d_off_x0020_status">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="24" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="25" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="26" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="442af37a-3796-4d85-82a9-7fed4a3d9bab" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="12" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c01f1a95-fe8a-4ef2-a1aa-bea3be48d6af}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="442af37a-3796-4d85-82a9-7fed4a3d9bab">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="16" nillable="true" ma:displayName="Compartilhado com" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="17" nillable="true" ma:displayName="Detalhes de Compartilhado Com" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de Conteúdo"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b633a64c-250e-4f9b-b03e-91a68bc51404">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <TaxCatchAll xmlns="442af37a-3796-4d85-82a9-7fed4a3d9bab" xsi:nil="true"/>
+    <_Flow_SignoffStatus xmlns="b633a64c-250e-4f9b-b03e-91a68bc51404" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CE3A740B-A3FE-4C50-A000-9FAE2510E700}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="b633a64c-250e-4f9b-b03e-91a68bc51404"/>
+    <ds:schemaRef ds:uri="442af37a-3796-4d85-82a9-7fed4a3d9bab"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BBBCA61A-72EE-4D20-B5D5-B108D9E4C84F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="b633a64c-250e-4f9b-b03e-91a68bc51404"/>
+    <ds:schemaRef ds:uri="442af37a-3796-4d85-82a9-7fed4a3d9bab"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5F9301C3-A4EA-4724-ABB3-5F8D135D20EC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Atualiza Gestão de Pendências · 2026-08-04T15:04:11.912-03:00
Responsável: Ana Paula da Mata Dias
</commit_message>
<xml_diff>
--- a/Base_Pendencias_FICO.xlsx
+++ b/Base_Pendencias_FICO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://globalvale.sharepoint.com/sites/PlanejamentoFICO/Shared Documents/General/04. Rotinas de desempenho FICO/06_Central de Acesso - Atualização/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="119" documentId="13_ncr:1_{9A6A02AB-2EB7-44B2-A1F8-27858C4205F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E4681AB2-670D-4289-A271-DBFDD627E6B6}"/>
+  <xr:revisionPtr revIDLastSave="174" documentId="13_ncr:1_{9A6A02AB-2EB7-44B2-A1F8-27858C4205F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1B38A9A2-2398-4F4C-8666-D41E2881341A}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INSTRUCOES" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="122">
   <si>
     <t>PAINEL DE PENDÊNCIAS FICO INFRA — BASE ÚNICA DE DADOS</t>
   </si>
@@ -220,15 +220,9 @@
     <t>HIDRO</t>
   </si>
   <si>
-    <t>MARCO FINAL ATÉ 15/10</t>
-  </si>
-  <si>
     <t>VALE</t>
   </si>
   <si>
-    <t>Em definição</t>
-  </si>
-  <si>
     <t>REPAROS</t>
   </si>
   <si>
@@ -410,6 +404,12 @@
   </si>
   <si>
     <t>15/10/2026 — Hidro e TAC 05 (Pacote 01)</t>
+  </si>
+  <si>
+    <t>Não será realizado pela EMPA</t>
+  </si>
+  <si>
+    <t>Marco final - 30/09/26</t>
   </si>
 </sst>
 </file>
@@ -557,7 +557,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -600,6 +600,19 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -685,6 +698,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -867,95 +884,95 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:B20"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
     <col min="2" max="2" width="115" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:2" ht="21" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:2" ht="20.25" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B3" s="2"/>
     </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B4" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B5" s="2"/>
     </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B6" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B10" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B11" s="2"/>
     </row>
-    <row r="12" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B12" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B13" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B15" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B16" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18" s="2"/>
     </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B19" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B20" s="2" t="s">
         <v>14</v>
       </c>
@@ -969,27 +986,27 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:P4"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="5.109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="17.44140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="19.109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="44.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="44.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>15</v>
       </c>
@@ -1039,7 +1056,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>31</v>
       </c>
@@ -1089,7 +1106,7 @@
       </c>
       <c r="P2" s="7"/>
     </row>
-    <row r="3" spans="1:16" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>38</v>
       </c>
@@ -1112,14 +1129,14 @@
         <v>29</v>
       </c>
       <c r="H3" s="9">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="I3" s="9">
         <v>60</v>
       </c>
       <c r="J3" s="6">
         <f>IF(I3=0,0,ROUND((1-H3/I3)*100,0))</f>
-        <v>50</v>
+        <v>82</v>
       </c>
       <c r="K3" s="7" t="s">
         <v>35</v>
@@ -1140,7 +1157,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>45</v>
       </c>
@@ -1197,19 +1214,19 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:K14"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="32.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="32.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>15</v>
       </c>
@@ -1232,7 +1249,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>31</v>
       </c>
@@ -1243,18 +1260,18 @@
         <v>56</v>
       </c>
       <c r="D2" s="6">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E2" s="8">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F2" s="10">
-        <f t="shared" ref="F2:F11" si="0">D2-E2</f>
-        <v>43</v>
+        <f t="shared" ref="F2:F13" si="0">D2-E2</f>
+        <v>39</v>
       </c>
       <c r="G2" s="7"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>31</v>
       </c>
@@ -1265,20 +1282,20 @@
         <v>57</v>
       </c>
       <c r="D3" s="6">
-        <v>111</v>
+        <v>79</v>
       </c>
       <c r="E3" s="8">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F3" s="10">
         <f t="shared" si="0"/>
-        <v>101</v>
+        <v>73</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>31</v>
       </c>
@@ -1289,154 +1306,157 @@
         <v>59</v>
       </c>
       <c r="D4" s="6">
-        <v>101</v>
+        <v>661</v>
       </c>
       <c r="E4" s="8">
-        <v>1</v>
+        <v>307</v>
       </c>
       <c r="F4" s="10">
         <f t="shared" si="0"/>
-        <v>100</v>
+        <v>354</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+        <v>121</v>
+      </c>
+      <c r="I4" s="18"/>
+      <c r="J4" s="18"/>
+      <c r="K4" s="18"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>31</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>32</v>
+        <v>58</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D5" s="6">
-        <v>83</v>
+        <v>13</v>
       </c>
       <c r="E5" s="8">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="F5" s="10">
         <f t="shared" si="0"/>
-        <v>48</v>
+        <v>13</v>
       </c>
       <c r="G5" s="7"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="D6" s="6">
+        <v>88</v>
+      </c>
+      <c r="E6" s="8">
+        <v>1</v>
+      </c>
+      <c r="F6" s="10">
+        <f t="shared" ref="F6" si="1">D6-E6</f>
+        <v>87</v>
+      </c>
+      <c r="G6" s="7"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B7" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C7" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="D6" s="6">
-        <v>37</v>
-      </c>
-      <c r="E6" s="8">
-        <v>9</v>
-      </c>
-      <c r="F6" s="10">
+      <c r="D7" s="6">
+        <v>53</v>
+      </c>
+      <c r="E7" s="8">
+        <v>25</v>
+      </c>
+      <c r="F7" s="10">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="G6" s="7"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="6" t="s">
+      <c r="G7" s="7"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B8" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C8" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="D7" s="6">
-        <v>39</v>
-      </c>
-      <c r="E7" s="8">
-        <v>2</v>
-      </c>
-      <c r="F7" s="10">
+      <c r="D8" s="6">
+        <v>40</v>
+      </c>
+      <c r="E8" s="8">
+        <v>3</v>
+      </c>
+      <c r="F8" s="10">
         <f t="shared" si="0"/>
         <v>37</v>
       </c>
-      <c r="G7" s="7"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="6" t="s">
+      <c r="G8" s="7"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B9" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C8" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="D8" s="6">
-        <v>114</v>
-      </c>
-      <c r="E8" s="8">
-        <v>23</v>
-      </c>
-      <c r="F8" s="10">
-        <f t="shared" si="0"/>
-        <v>91</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>46</v>
-      </c>
       <c r="C9" s="7" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="D9" s="6">
-        <v>33</v>
+        <v>634</v>
       </c>
       <c r="E9" s="8">
-        <v>2</v>
+        <v>167</v>
       </c>
       <c r="F9" s="10">
         <f t="shared" si="0"/>
-        <v>31</v>
-      </c>
-      <c r="G9" s="7"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+        <v>467</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D10" s="6">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="E10" s="8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F10" s="10">
         <f t="shared" si="0"/>
-        <v>48</v>
+        <v>10</v>
       </c>
       <c r="G10" s="7"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>45</v>
       </c>
@@ -1444,21 +1464,87 @@
         <v>46</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="D11" s="6">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E11" s="8">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="F11" s="10">
         <f t="shared" si="0"/>
-        <v>32</v>
-      </c>
-      <c r="G11" s="7" t="s">
-        <v>63</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="G11" s="7"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="D12" s="6">
+        <v>100</v>
+      </c>
+      <c r="E12" s="8">
+        <v>5</v>
+      </c>
+      <c r="F12" s="10">
+        <f t="shared" si="0"/>
+        <v>95</v>
+      </c>
+      <c r="G12" s="7"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="D13" s="6">
+        <v>839</v>
+      </c>
+      <c r="E13" s="8">
+        <v>155</v>
+      </c>
+      <c r="F13" s="10">
+        <f t="shared" si="0"/>
+        <v>684</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="B14" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="C14" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="D14" s="19">
+        <v>14</v>
+      </c>
+      <c r="E14" s="21">
+        <v>0</v>
+      </c>
+      <c r="F14" s="22">
+        <f t="shared" ref="F14" si="2">D14-E14</f>
+        <v>14</v>
+      </c>
+      <c r="G14" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1469,45 +1555,45 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>15</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>66</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>68</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>23</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>31</v>
       </c>
@@ -1524,12 +1610,12 @@
         <v>12</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G2" s="6"/>
       <c r="H2" s="7"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>31</v>
       </c>
@@ -1549,7 +1635,7 @@
       <c r="G3" s="6"/>
       <c r="H3" s="7"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>31</v>
       </c>
@@ -1567,11 +1653,11 @@
       </c>
       <c r="F4" s="6"/>
       <c r="G4" s="6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="H4" s="7"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>31</v>
       </c>
@@ -1591,7 +1677,7 @@
       <c r="G5" s="6"/>
       <c r="H5" s="7"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>38</v>
       </c>
@@ -1611,7 +1697,7 @@
       <c r="G6" s="6"/>
       <c r="H6" s="7"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>38</v>
       </c>
@@ -1628,12 +1714,12 @@
         <v>36</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G7" s="6"/>
       <c r="H7" s="7"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>38</v>
       </c>
@@ -1653,7 +1739,7 @@
       <c r="G8" s="6"/>
       <c r="H8" s="7"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>45</v>
       </c>
@@ -1671,11 +1757,11 @@
       </c>
       <c r="F9" s="6"/>
       <c r="G9" s="6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="H9" s="7"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>45</v>
       </c>
@@ -1695,7 +1781,7 @@
       <c r="G10" s="6"/>
       <c r="H10" s="7"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>45</v>
       </c>
@@ -1724,15 +1810,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="38.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="84.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="84.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>15</v>
       </c>
@@ -1740,234 +1826,234 @@
         <v>51</v>
       </c>
       <c r="C1" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="B2" s="11" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A2" s="10" t="s">
+      <c r="C2" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="D2" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="C2" s="12" t="s">
+    </row>
+    <row r="3" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A3" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="B3" s="13" t="s">
         <v>75</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="C3" s="12" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A3" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="B3" s="13" t="s">
+      <c r="D3" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="C3" s="12" t="s">
+    </row>
+    <row r="4" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A4" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="B4" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="C4" s="12" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A4" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="B4" s="14" t="s">
+      <c r="D4" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="C4" s="12" t="s">
+    </row>
+    <row r="5" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A5" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="B5" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="C5" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D5" s="7" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A5" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="B5" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="C5" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>31</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>31</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>31</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>31</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
         <v>38</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
         <v>38</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
         <v>38</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
         <v>38</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A14" s="10" t="s">
         <v>45</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
         <v>45</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A16" s="10" t="s">
         <v>45</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
         <v>45</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>
@@ -1979,66 +2065,66 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="B1" s="5" t="s">
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="15" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="B2" s="7" t="s">
+      <c r="B3" s="7" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="15" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B4" s="16" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" s="15" t="s">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="B4" s="16" t="s">
+      <c r="B5" s="7" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" s="15" t="s">
+    <row r="6" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A6" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B6" s="7" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="15" t="s">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="15" t="s">
         <v>118</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B7" s="7" t="s">
         <v>119</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" s="15" t="s">
-        <v>120</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -2312,6 +2398,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="b633a64c-250e-4f9b-b03e-91a68bc51404">
@@ -2323,15 +2418,6 @@
     <_Flow_SignoffStatus xmlns="b633a64c-250e-4f9b-b03e-91a68bc51404" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2355,6 +2441,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5F9301C3-A4EA-4724-ABB3-5F8D135D20EC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BBBCA61A-72EE-4D20-B5D5-B108D9E4C84F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
@@ -2372,14 +2466,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5F9301C3-A4EA-4724-ABB3-5F8D135D20EC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{340ed6a7-0f03-43d9-901d-02d4a7e408aa}" enabled="1" method="Privileged" siteId="{7893571b-6c2c-4cef-b4da-7d4b266a0626}" contentBits="0" removed="0"/>

</xml_diff>

<commit_message>
Atualiza Gestão de Pendências · 2026-08-04T16:24:10.614-03:00
Responsável: Ana Paula da Mata Dias
</commit_message>
<xml_diff>
--- a/Base_Pendencias_FICO.xlsx
+++ b/Base_Pendencias_FICO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://globalvale.sharepoint.com/sites/PlanejamentoFICO/Shared Documents/General/04. Rotinas de desempenho FICO/06_Central de Acesso - Atualização/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="174" documentId="13_ncr:1_{9A6A02AB-2EB7-44B2-A1F8-27858C4205F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1B38A9A2-2398-4F4C-8666-D41E2881341A}"/>
+  <xr:revisionPtr revIDLastSave="175" documentId="13_ncr:1_{9A6A02AB-2EB7-44B2-A1F8-27858C4205F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6246E5FE-DB9B-4A5F-9ADC-0F6F001B4425}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INSTRUCOES" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <sheet name="ALERTAS" sheetId="5" r:id="rId5"/>
     <sheet name="META" sheetId="6" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191028" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="121">
   <si>
     <t>PAINEL DE PENDÊNCIAS FICO INFRA — BASE ÚNICA DE DADOS</t>
   </si>
@@ -383,9 +383,6 @@
   </si>
   <si>
     <t>DATA_REFERENCIA</t>
-  </si>
-  <si>
-    <t>07/07/2026</t>
   </si>
   <si>
     <t>CADENCIA</t>
@@ -557,7 +554,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -600,19 +597,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -698,10 +682,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1214,7 +1194,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
@@ -1226,7 +1206,7 @@
     <col min="7" max="7" width="32.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>15</v>
       </c>
@@ -1249,7 +1229,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>31</v>
       </c>
@@ -1271,7 +1251,7 @@
       </c>
       <c r="G2" s="7"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>31</v>
       </c>
@@ -1292,10 +1272,10 @@
         <v>73</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>31</v>
       </c>
@@ -1316,13 +1296,10 @@
         <v>354</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="I4" s="18"/>
-      <c r="J4" s="18"/>
-      <c r="K4" s="18"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>31</v>
       </c>
@@ -1344,7 +1321,7 @@
       </c>
       <c r="G5" s="7"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>31</v>
       </c>
@@ -1366,7 +1343,7 @@
       </c>
       <c r="G6" s="7"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>38</v>
       </c>
@@ -1388,7 +1365,7 @@
       </c>
       <c r="G7" s="7"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>38</v>
       </c>
@@ -1410,7 +1387,7 @@
       </c>
       <c r="G8" s="7"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>38</v>
       </c>
@@ -1434,7 +1411,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>38</v>
       </c>
@@ -1456,7 +1433,7 @@
       </c>
       <c r="G10" s="7"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>45</v>
       </c>
@@ -1478,7 +1455,7 @@
       </c>
       <c r="G11" s="7"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>45</v>
       </c>
@@ -1500,7 +1477,7 @@
       </c>
       <c r="G12" s="7"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>45</v>
       </c>
@@ -1524,23 +1501,23 @@
         <v>61</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="19" t="s">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="B14" s="20" t="s">
+      <c r="B14" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="C14" s="20" t="s">
+      <c r="C14" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="D14" s="19">
+      <c r="D14" s="6">
         <v>14</v>
       </c>
-      <c r="E14" s="21">
+      <c r="E14" s="8">
         <v>0</v>
       </c>
-      <c r="F14" s="22">
+      <c r="F14" s="10">
         <f t="shared" ref="F14" si="2">D14-E14</f>
         <v>14</v>
       </c>
@@ -2099,32 +2076,32 @@
       <c r="A4" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="B4" s="16" t="s">
-        <v>113</v>
+      <c r="B4" s="16">
+        <v>46238</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
+        <v>113</v>
+      </c>
+      <c r="B5" s="7" t="s">
         <v>114</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="B6" s="7" t="s">
         <v>116</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="B7" s="7" t="s">
         <v>118</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -2134,6 +2111,29 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b633a64c-250e-4f9b-b03e-91a68bc51404">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <TaxCatchAll xmlns="442af37a-3796-4d85-82a9-7fed4a3d9bab" xsi:nil="true"/>
+    <_Flow_SignoffStatus xmlns="b633a64c-250e-4f9b-b03e-91a68bc51404" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100401A7D55F60B18408D7825C28E029F51" ma:contentTypeVersion="19" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="26245b19684232a249215bac47317027">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="b633a64c-250e-4f9b-b03e-91a68bc51404" xmlns:ns3="442af37a-3796-4d85-82a9-7fed4a3d9bab" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0b8051d1477f5ab751da8276506a6b46" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -2397,30 +2397,33 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BBBCA61A-72EE-4D20-B5D5-B108D9E4C84F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="442af37a-3796-4d85-82a9-7fed4a3d9bab"/>
+    <ds:schemaRef ds:uri="b633a64c-250e-4f9b-b03e-91a68bc51404"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b633a64c-250e-4f9b-b03e-91a68bc51404">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <TaxCatchAll xmlns="442af37a-3796-4d85-82a9-7fed4a3d9bab" xsi:nil="true"/>
-    <_Flow_SignoffStatus xmlns="b633a64c-250e-4f9b-b03e-91a68bc51404" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5F9301C3-A4EA-4724-ABB3-5F8D135D20EC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CE3A740B-A3FE-4C50-A000-9FAE2510E700}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2440,32 +2443,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5F9301C3-A4EA-4724-ABB3-5F8D135D20EC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BBBCA61A-72EE-4D20-B5D5-B108D9E4C84F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="b633a64c-250e-4f9b-b03e-91a68bc51404"/>
-    <ds:schemaRef ds:uri="442af37a-3796-4d85-82a9-7fed4a3d9bab"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{340ed6a7-0f03-43d9-901d-02d4a7e408aa}" enabled="1" method="Privileged" siteId="{7893571b-6c2c-4cef-b4da-7d4b266a0626}" contentBits="0" removed="0"/>

</xml_diff>

<commit_message>
Atualiza Gestão de Pendências · 2026-08-05T08:07:23.909-03:00
Responsável: Ana Paula da Mata Dias
</commit_message>
<xml_diff>
--- a/Base_Pendencias_FICO.xlsx
+++ b/Base_Pendencias_FICO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://globalvale.sharepoint.com/sites/PlanejamentoFICO/Shared Documents/General/04. Rotinas de desempenho FICO/06_Central de Acesso - Atualização/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="175" documentId="13_ncr:1_{9A6A02AB-2EB7-44B2-A1F8-27858C4205F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6246E5FE-DB9B-4A5F-9ADC-0F6F001B4425}"/>
+  <xr:revisionPtr revIDLastSave="184" documentId="13_ncr:1_{9A6A02AB-2EB7-44B2-A1F8-27858C4205F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{539361F0-69F5-4364-9701-9B948BDFDFE3}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="122">
   <si>
     <t>PAINEL DE PENDÊNCIAS FICO INFRA — BASE ÚNICA DE DADOS</t>
   </si>
@@ -407,6 +407,9 @@
   </si>
   <si>
     <t>Marco final - 30/09/26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">04/08/2026 </t>
   </si>
 </sst>
 </file>
@@ -593,11 +596,11 @@
     <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="1" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1577,10 +1580,10 @@
       <c r="B2" s="10">
         <v>1</v>
       </c>
-      <c r="C2" s="17">
+      <c r="C2" s="16">
         <v>5.375</v>
       </c>
-      <c r="D2" s="17">
+      <c r="D2" s="16">
         <v>1.075</v>
       </c>
       <c r="E2" s="6">
@@ -1599,10 +1602,10 @@
       <c r="B3" s="10">
         <v>2</v>
       </c>
-      <c r="C3" s="17">
+      <c r="C3" s="16">
         <v>12.625</v>
       </c>
-      <c r="D3" s="17">
+      <c r="D3" s="16">
         <v>2.5249999999999999</v>
       </c>
       <c r="E3" s="6">
@@ -1619,10 +1622,10 @@
       <c r="B4" s="10">
         <v>3</v>
       </c>
-      <c r="C4" s="17">
+      <c r="C4" s="16">
         <v>12.5</v>
       </c>
-      <c r="D4" s="17">
+      <c r="D4" s="16">
         <v>2.5</v>
       </c>
       <c r="E4" s="6">
@@ -1641,10 +1644,10 @@
       <c r="B5" s="10">
         <v>1</v>
       </c>
-      <c r="C5" s="17">
+      <c r="C5" s="16">
         <v>6</v>
       </c>
-      <c r="D5" s="17">
+      <c r="D5" s="16">
         <v>1.2</v>
       </c>
       <c r="E5" s="6">
@@ -1661,10 +1664,10 @@
       <c r="B6" s="10">
         <v>2</v>
       </c>
-      <c r="C6" s="17">
+      <c r="C6" s="16">
         <v>3.5</v>
       </c>
-      <c r="D6" s="17">
+      <c r="D6" s="16">
         <v>0.7</v>
       </c>
       <c r="E6" s="6">
@@ -1681,10 +1684,10 @@
       <c r="B7" s="10">
         <v>3</v>
       </c>
-      <c r="C7" s="17">
+      <c r="C7" s="16">
         <v>4.625</v>
       </c>
-      <c r="D7" s="17">
+      <c r="D7" s="16">
         <v>0.92500000000000004</v>
       </c>
       <c r="E7" s="6">
@@ -1703,10 +1706,10 @@
       <c r="B8" s="10">
         <v>4</v>
       </c>
-      <c r="C8" s="17">
+      <c r="C8" s="16">
         <v>11.375</v>
       </c>
-      <c r="D8" s="17">
+      <c r="D8" s="16">
         <v>2.2749999999999999</v>
       </c>
       <c r="E8" s="6">
@@ -1723,10 +1726,10 @@
       <c r="B9" s="10">
         <v>5</v>
       </c>
-      <c r="C9" s="17">
+      <c r="C9" s="16">
         <v>3.875</v>
       </c>
-      <c r="D9" s="17">
+      <c r="D9" s="16">
         <v>0.77500000000000002</v>
       </c>
       <c r="E9" s="6">
@@ -1745,10 +1748,10 @@
       <c r="B10" s="10">
         <v>1</v>
       </c>
-      <c r="C10" s="17">
+      <c r="C10" s="16">
         <v>6</v>
       </c>
-      <c r="D10" s="17">
+      <c r="D10" s="16">
         <v>1.2</v>
       </c>
       <c r="E10" s="6">
@@ -1765,10 +1768,10 @@
       <c r="B11" s="10">
         <v>2</v>
       </c>
-      <c r="C11" s="17">
+      <c r="C11" s="16">
         <v>4</v>
       </c>
-      <c r="D11" s="17">
+      <c r="D11" s="16">
         <v>0.8</v>
       </c>
       <c r="E11" s="6">
@@ -2076,8 +2079,8 @@
       <c r="A4" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="B4" s="16">
-        <v>46238</v>
+      <c r="B4" s="17" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -2111,29 +2114,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b633a64c-250e-4f9b-b03e-91a68bc51404">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <TaxCatchAll xmlns="442af37a-3796-4d85-82a9-7fed4a3d9bab" xsi:nil="true"/>
-    <_Flow_SignoffStatus xmlns="b633a64c-250e-4f9b-b03e-91a68bc51404" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100401A7D55F60B18408D7825C28E029F51" ma:contentTypeVersion="19" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="26245b19684232a249215bac47317027">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="b633a64c-250e-4f9b-b03e-91a68bc51404" xmlns:ns3="442af37a-3796-4d85-82a9-7fed4a3d9bab" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0b8051d1477f5ab751da8276506a6b46" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -2397,33 +2377,30 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BBBCA61A-72EE-4D20-B5D5-B108D9E4C84F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="442af37a-3796-4d85-82a9-7fed4a3d9bab"/>
-    <ds:schemaRef ds:uri="b633a64c-250e-4f9b-b03e-91a68bc51404"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5F9301C3-A4EA-4724-ABB3-5F8D135D20EC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b633a64c-250e-4f9b-b03e-91a68bc51404">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <TaxCatchAll xmlns="442af37a-3796-4d85-82a9-7fed4a3d9bab" xsi:nil="true"/>
+    <_Flow_SignoffStatus xmlns="b633a64c-250e-4f9b-b03e-91a68bc51404" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CE3A740B-A3FE-4C50-A000-9FAE2510E700}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2443,6 +2420,32 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5F9301C3-A4EA-4724-ABB3-5F8D135D20EC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BBBCA61A-72EE-4D20-B5D5-B108D9E4C84F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="442af37a-3796-4d85-82a9-7fed4a3d9bab"/>
+    <ds:schemaRef ds:uri="b633a64c-250e-4f9b-b03e-91a68bc51404"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{340ed6a7-0f03-43d9-901d-02d4a7e408aa}" enabled="1" method="Privileged" siteId="{7893571b-6c2c-4cef-b4da-7d4b266a0626}" contentBits="0" removed="0"/>

</xml_diff>

<commit_message>
Atualiza Gestão de Pendências · 2026-08-11T18:12:09.764-03:00
Responsável: Eder Valasco
</commit_message>
<xml_diff>
--- a/Base_Pendencias_FICO.xlsx
+++ b/Base_Pendencias_FICO.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://globalvale.sharepoint.com/sites/PlanejamentoFICO/Shared Documents/General/04. Rotinas de desempenho FICO/06_Central de Acesso - Atualização/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\valasede\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="184" documentId="13_ncr:1_{9A6A02AB-2EB7-44B2-A1F8-27858C4205F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{539361F0-69F5-4364-9701-9B948BDFDFE3}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{571DECB2-F965-4011-83BF-97733BA689AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INSTRUCOES" sheetId="1" r:id="rId1"/>
@@ -409,7 +409,7 @@
     <t>Marco final - 30/09/26</t>
   </si>
   <si>
-    <t xml:space="preserve">04/08/2026 </t>
+    <t xml:space="preserve">11/08/2026 </t>
   </si>
 </sst>
 </file>
@@ -599,7 +599,7 @@
     <xf numFmtId="1" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -867,95 +867,95 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:B20"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
     <col min="2" max="2" width="115" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:2" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:2" ht="20" x14ac:dyDescent="0.4">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B3" s="2"/>
     </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B5" s="2"/>
     </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B6" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B7" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B8" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B9" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B10" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B11" s="2"/>
     </row>
-    <row r="12" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B12" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B13" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B14" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B15" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B16" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B17" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B18" s="2"/>
     </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B19" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B20" s="2" t="s">
         <v>14</v>
       </c>
@@ -969,27 +969,27 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:P4"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.453125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="5.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="44.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.7265625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.1796875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="19.1796875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="44.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" ht="27" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>15</v>
       </c>
@@ -1039,7 +1039,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" ht="25" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
         <v>31</v>
       </c>
@@ -1089,7 +1089,7 @@
       </c>
       <c r="P2" s="7"/>
     </row>
-    <row r="3" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" ht="25" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
         <v>38</v>
       </c>
@@ -1140,7 +1140,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" ht="25" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
         <v>45</v>
       </c>
@@ -1198,18 +1198,18 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:G14"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="32.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="32.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>15</v>
       </c>
@@ -1232,7 +1232,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
         <v>31</v>
       </c>
@@ -1246,15 +1246,15 @@
         <v>84</v>
       </c>
       <c r="E2" s="8">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F2" s="10">
         <f t="shared" ref="F2:F13" si="0">D2-E2</f>
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G2" s="7"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
         <v>31</v>
       </c>
@@ -1265,20 +1265,20 @@
         <v>57</v>
       </c>
       <c r="D3" s="6">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E3" s="8">
         <v>6</v>
       </c>
       <c r="F3" s="10">
         <f t="shared" si="0"/>
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G3" s="7" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
         <v>31</v>
       </c>
@@ -1289,20 +1289,20 @@
         <v>59</v>
       </c>
       <c r="D4" s="6">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="E4" s="8">
-        <v>307</v>
+        <v>340</v>
       </c>
       <c r="F4" s="10">
         <f t="shared" si="0"/>
-        <v>354</v>
+        <v>319</v>
       </c>
       <c r="G4" s="7" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
         <v>31</v>
       </c>
@@ -1324,7 +1324,7 @@
       </c>
       <c r="G5" s="7"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
         <v>31</v>
       </c>
@@ -1346,7 +1346,7 @@
       </c>
       <c r="G6" s="7"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
         <v>38</v>
       </c>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="G7" s="7"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
         <v>38</v>
       </c>
@@ -1390,7 +1390,7 @@
       </c>
       <c r="G8" s="7"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
         <v>38</v>
       </c>
@@ -1401,20 +1401,20 @@
         <v>59</v>
       </c>
       <c r="D9" s="6">
-        <v>634</v>
+        <v>630</v>
       </c>
       <c r="E9" s="8">
-        <v>167</v>
+        <v>191</v>
       </c>
       <c r="F9" s="10">
         <f t="shared" si="0"/>
-        <v>467</v>
+        <v>439</v>
       </c>
       <c r="G9" s="7" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="6" t="s">
         <v>38</v>
       </c>
@@ -1425,18 +1425,18 @@
         <v>59</v>
       </c>
       <c r="D10" s="6">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E10" s="8">
         <v>0</v>
       </c>
       <c r="F10" s="10">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G10" s="7"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
         <v>45</v>
       </c>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="G11" s="7"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="6" t="s">
         <v>45</v>
       </c>
@@ -1472,15 +1472,15 @@
         <v>100</v>
       </c>
       <c r="E12" s="8">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F12" s="10">
         <f t="shared" si="0"/>
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="G12" s="7"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="6" t="s">
         <v>45</v>
       </c>
@@ -1491,20 +1491,20 @@
         <v>59</v>
       </c>
       <c r="D13" s="6">
-        <v>839</v>
+        <v>819</v>
       </c>
       <c r="E13" s="8">
-        <v>155</v>
+        <v>211</v>
       </c>
       <c r="F13" s="10">
         <f t="shared" si="0"/>
-        <v>684</v>
+        <v>608</v>
       </c>
       <c r="G13" s="7" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="6" t="s">
         <v>45</v>
       </c>
@@ -1535,19 +1535,19 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>15</v>
       </c>
@@ -1573,7 +1573,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
         <v>31</v>
       </c>
@@ -1581,13 +1581,13 @@
         <v>1</v>
       </c>
       <c r="C2" s="16">
-        <v>5.375</v>
+        <v>5.4285714285714288</v>
       </c>
       <c r="D2" s="16">
         <v>1.075</v>
       </c>
-      <c r="E2" s="6">
-        <v>12</v>
+      <c r="E2" s="16">
+        <v>1.0857142857142859</v>
       </c>
       <c r="F2" s="6" t="s">
         <v>68</v>
@@ -1595,7 +1595,7 @@
       <c r="G2" s="6"/>
       <c r="H2" s="7"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
         <v>31</v>
       </c>
@@ -1603,19 +1603,19 @@
         <v>2</v>
       </c>
       <c r="C3" s="16">
-        <v>12.625</v>
+        <v>10.285714285714286</v>
       </c>
       <c r="D3" s="16">
         <v>2.5249999999999999</v>
       </c>
-      <c r="E3" s="6">
-        <v>24</v>
+      <c r="E3" s="16">
+        <v>2.0571428571428574</v>
       </c>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
       <c r="H3" s="7"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
         <v>31</v>
       </c>
@@ -1623,13 +1623,13 @@
         <v>3</v>
       </c>
       <c r="C4" s="16">
-        <v>12.5</v>
+        <v>45.571428571428569</v>
       </c>
       <c r="D4" s="16">
         <v>2.5</v>
       </c>
-      <c r="E4" s="6">
-        <v>36</v>
+      <c r="E4" s="16">
+        <v>9.1142857142857139</v>
       </c>
       <c r="F4" s="6"/>
       <c r="G4" s="6" t="s">
@@ -1637,7 +1637,7 @@
       </c>
       <c r="H4" s="7"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
         <v>31</v>
       </c>
@@ -1645,19 +1645,19 @@
         <v>1</v>
       </c>
       <c r="C5" s="16">
-        <v>6</v>
+        <v>1.8571428571428572</v>
       </c>
       <c r="D5" s="16">
         <v>1.2</v>
       </c>
-      <c r="E5" s="6">
-        <v>12</v>
+      <c r="E5" s="16">
+        <v>0.37142857142857144</v>
       </c>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
       <c r="H5" s="7"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
         <v>38</v>
       </c>
@@ -1665,19 +1665,19 @@
         <v>2</v>
       </c>
       <c r="C6" s="16">
-        <v>3.5</v>
+        <v>12.428571428571429</v>
       </c>
       <c r="D6" s="16">
         <v>0.7</v>
       </c>
-      <c r="E6" s="6">
-        <v>24</v>
+      <c r="E6" s="16">
+        <v>2.4857142857142858</v>
       </c>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
       <c r="H6" s="7"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
         <v>38</v>
       </c>
@@ -1685,13 +1685,13 @@
         <v>3</v>
       </c>
       <c r="C7" s="16">
-        <v>4.625</v>
+        <v>4</v>
       </c>
       <c r="D7" s="16">
         <v>0.92500000000000004</v>
       </c>
-      <c r="E7" s="6">
-        <v>36</v>
+      <c r="E7" s="16">
+        <v>0.8</v>
       </c>
       <c r="F7" s="6" t="s">
         <v>68</v>
@@ -1699,7 +1699,7 @@
       <c r="G7" s="6"/>
       <c r="H7" s="7"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
         <v>38</v>
       </c>
@@ -1707,19 +1707,19 @@
         <v>4</v>
       </c>
       <c r="C8" s="16">
-        <v>11.375</v>
+        <v>5.2857142857142856</v>
       </c>
       <c r="D8" s="16">
         <v>2.2749999999999999</v>
       </c>
-      <c r="E8" s="6">
-        <v>48</v>
+      <c r="E8" s="16">
+        <v>1.0571428571428572</v>
       </c>
       <c r="F8" s="6"/>
       <c r="G8" s="6"/>
       <c r="H8" s="7"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
         <v>45</v>
       </c>
@@ -1727,13 +1727,13 @@
         <v>5</v>
       </c>
       <c r="C9" s="16">
-        <v>3.875</v>
+        <v>62.714285714285715</v>
       </c>
       <c r="D9" s="16">
         <v>0.77500000000000002</v>
       </c>
-      <c r="E9" s="6">
-        <v>60</v>
+      <c r="E9" s="16">
+        <v>12.542857142857143</v>
       </c>
       <c r="F9" s="6"/>
       <c r="G9" s="6" t="s">
@@ -1741,7 +1741,7 @@
       </c>
       <c r="H9" s="7"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="6" t="s">
         <v>45</v>
       </c>
@@ -1749,19 +1749,19 @@
         <v>1</v>
       </c>
       <c r="C10" s="16">
-        <v>6</v>
+        <v>1.1428571428571428</v>
       </c>
       <c r="D10" s="16">
         <v>1.2</v>
       </c>
-      <c r="E10" s="6">
-        <v>12</v>
+      <c r="E10" s="16">
+        <v>0.22857142857142856</v>
       </c>
       <c r="F10" s="6"/>
       <c r="G10" s="6"/>
       <c r="H10" s="7"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
         <v>45</v>
       </c>
@@ -1769,13 +1769,13 @@
         <v>2</v>
       </c>
       <c r="C11" s="16">
-        <v>4</v>
+        <v>5.8571428571428568</v>
       </c>
       <c r="D11" s="16">
         <v>0.8</v>
       </c>
-      <c r="E11" s="6">
-        <v>24</v>
+      <c r="E11" s="16">
+        <v>1.1714285714285713</v>
       </c>
       <c r="F11" s="6"/>
       <c r="G11" s="6"/>
@@ -1790,15 +1790,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="38.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="84.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="84.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>15</v>
       </c>
@@ -1812,7 +1812,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ht="25" x14ac:dyDescent="0.35">
       <c r="A2" s="10" t="s">
         <v>71</v>
       </c>
@@ -1826,7 +1826,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" ht="25" x14ac:dyDescent="0.35">
       <c r="A3" s="10" t="s">
         <v>71</v>
       </c>
@@ -1840,7 +1840,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" ht="25" x14ac:dyDescent="0.35">
       <c r="A4" s="10" t="s">
         <v>71</v>
       </c>
@@ -1854,7 +1854,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" ht="25" x14ac:dyDescent="0.35">
       <c r="A5" s="10" t="s">
         <v>71</v>
       </c>
@@ -1868,7 +1868,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" ht="25" x14ac:dyDescent="0.35">
       <c r="A6" s="10" t="s">
         <v>31</v>
       </c>
@@ -1882,7 +1882,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" ht="25" x14ac:dyDescent="0.35">
       <c r="A7" s="10" t="s">
         <v>31</v>
       </c>
@@ -1896,7 +1896,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" ht="25" x14ac:dyDescent="0.35">
       <c r="A8" s="10" t="s">
         <v>31</v>
       </c>
@@ -1910,7 +1910,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="10" t="s">
         <v>31</v>
       </c>
@@ -1924,7 +1924,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" ht="25" x14ac:dyDescent="0.35">
       <c r="A10" s="10" t="s">
         <v>38</v>
       </c>
@@ -1938,7 +1938,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" ht="25" x14ac:dyDescent="0.35">
       <c r="A11" s="10" t="s">
         <v>38</v>
       </c>
@@ -1952,7 +1952,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" ht="25" x14ac:dyDescent="0.35">
       <c r="A12" s="10" t="s">
         <v>38</v>
       </c>
@@ -1966,7 +1966,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="10" t="s">
         <v>38</v>
       </c>
@@ -1980,7 +1980,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" ht="25" x14ac:dyDescent="0.35">
       <c r="A14" s="10" t="s">
         <v>45</v>
       </c>
@@ -1994,7 +1994,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" ht="25" x14ac:dyDescent="0.35">
       <c r="A15" s="10" t="s">
         <v>45</v>
       </c>
@@ -2008,7 +2008,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="10" t="s">
         <v>45</v>
       </c>
@@ -2022,7 +2022,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" ht="25" x14ac:dyDescent="0.35">
       <c r="A17" s="10" t="s">
         <v>45</v>
       </c>
@@ -2045,13 +2045,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>107</v>
       </c>
@@ -2059,7 +2059,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="15" t="s">
         <v>69</v>
       </c>
@@ -2067,7 +2067,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="15" t="s">
         <v>110</v>
       </c>
@@ -2075,7 +2075,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" s="15" t="s">
         <v>112</v>
       </c>
@@ -2083,7 +2083,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="15" t="s">
         <v>113</v>
       </c>
@@ -2091,7 +2091,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" ht="25" x14ac:dyDescent="0.35">
       <c r="A6" s="15" t="s">
         <v>115</v>
       </c>
@@ -2099,7 +2099,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" s="15" t="s">
         <v>117</v>
       </c>
@@ -2114,6 +2114,20 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b633a64c-250e-4f9b-b03e-91a68bc51404">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <TaxCatchAll xmlns="442af37a-3796-4d85-82a9-7fed4a3d9bab" xsi:nil="true"/>
+    <_Flow_SignoffStatus xmlns="b633a64c-250e-4f9b-b03e-91a68bc51404" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100401A7D55F60B18408D7825C28E029F51" ma:contentTypeVersion="19" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="26245b19684232a249215bac47317027">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="b633a64c-250e-4f9b-b03e-91a68bc51404" xmlns:ns3="442af37a-3796-4d85-82a9-7fed4a3d9bab" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0b8051d1477f5ab751da8276506a6b46" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -2377,7 +2391,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -2386,21 +2400,25 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b633a64c-250e-4f9b-b03e-91a68bc51404">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <TaxCatchAll xmlns="442af37a-3796-4d85-82a9-7fed4a3d9bab" xsi:nil="true"/>
-    <_Flow_SignoffStatus xmlns="b633a64c-250e-4f9b-b03e-91a68bc51404" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BBBCA61A-72EE-4D20-B5D5-B108D9E4C84F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="442af37a-3796-4d85-82a9-7fed4a3d9bab"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="b633a64c-250e-4f9b-b03e-91a68bc51404"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CE3A740B-A3FE-4C50-A000-9FAE2510E700}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2420,7 +2438,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5F9301C3-A4EA-4724-ABB3-5F8D135D20EC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -2428,26 +2446,8 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BBBCA61A-72EE-4D20-B5D5-B108D9E4C84F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="442af37a-3796-4d85-82a9-7fed4a3d9bab"/>
-    <ds:schemaRef ds:uri="b633a64c-250e-4f9b-b03e-91a68bc51404"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{340ed6a7-0f03-43d9-901d-02d4a7e408aa}" enabled="1" method="Privileged" siteId="{7893571b-6c2c-4cef-b4da-7d4b266a0626}" contentBits="0" removed="0"/>
+  <clbl:label id="{340ed6a7-0f03-43d9-901d-02d4a7e408aa}" enabled="1" method="Privileged" siteId="{7893571b-6c2c-4cef-b4da-7d4b266a0626}" removed="0"/>
 </clbl:labelList>
 </file>
</xml_diff>